<commit_message>
geração de relatório d inspeções
</commit_message>
<xml_diff>
--- a/dados/csv/inspecoes.xlsx
+++ b/dados/csv/inspecoes.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,76 +425,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>op</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>codigo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>data_hora_inicio_inspecao</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>data_hora_fim_inspecao</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>possui_op</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>qtd_etiquetas</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>conformidade</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>refugo</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>aprovado</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
@@ -516,12 +523,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-12T16:48:00</t>
+          <t>12/07/2026 16:48:00</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-07-12T16:49:00</t>
+          <t>12/07/2026 16:49:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -531,30 +538,25 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Conforme</t>
+          <t>True</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
         <is>
           <t>Item sem op</t>
         </is>
@@ -588,12 +590,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-14T14:36:00</t>
+          <t>14/07/2026 14:36:00</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-14T14:43:00</t>
+          <t>14/07/2026 14:43:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -603,30 +605,25 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>Não conforme</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>True</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
         <is>
           <t>Nao foi trocado a caixa de kit</t>
         </is>
@@ -660,12 +657,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-14T15:40:00</t>
+          <t>14/07/2026 15:40:00</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-14T15:53:00</t>
+          <t>14/07/2026 15:53:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -675,30 +672,25 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>Não conforme</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>True</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
         <is>
           <t>Motor faltando parafuso</t>
         </is>
@@ -732,12 +724,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-14T16:00:00</t>
+          <t>14/07/2026 16:00:00</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-14T16:02:00</t>
+          <t>14/07/2026 16:02:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -747,30 +739,25 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Conforme</t>
+          <t>True</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
         <is>
           <t>Capacitor de 30</t>
         </is>
@@ -804,12 +791,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-14T16:05:00</t>
+          <t>14/07/2026 16:05:00</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-07-14T16:12:00</t>
+          <t>14/07/2026 16:12:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -819,32 +806,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>Não conforme</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Não conforme</t>
+          <t>True</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>Motores sujos de PU e óleo 
+          <t>Motores sujos de PU e óleo 
 Etiqueta pivo na central pivo dupla</t>
         </is>
       </c>

</xml_diff>